<commit_message>
Categorisation script now analyses dataset and extracts all months covered. This is saved to a new metadata JSON file. Analysis script uses this and analyses spending/income per category/subcategory and per month. One table is created per month.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -827,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -844,168 +844,175 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>1825.6</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>-1825.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>1787.95</v>
+        <v>6966.35</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>23.95</v>
+        <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>1764</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>433.55</v>
+        <v>1825.6</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>-433.55</v>
+        <v>-1825.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Überträge</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>382.59</v>
+        <v>23.95</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>-382.59</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>130.5</v>
+        <v>433.55</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>-130.5</v>
+        <v>-433.55</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>382.59</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>-382.59</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>85</v>
+        <v>130.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>-85</v>
+        <v>-130.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>-85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="4" t="n">
+      <c r="B14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>12.4</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>-12.4</v>
       </c>
     </row>
@@ -1020,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1038,72 +1045,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Supermärkte</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>200.65</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>-200.65</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Detail-Lebensmittel</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>167.29</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>-167.29</v>
       </c>
     </row>
     <row r="6">
@@ -1114,143 +1086,143 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sonstiges Einkaufen</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>14.65</v>
+        <v>200.65</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>-14.65</v>
+        <v>-200.65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lohn</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>6966.35</v>
+        <v>0</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0</v>
+        <v>167.29</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>6966.35</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>80</v>
+        <v>14.65</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-80</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gebühren</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-5</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>130.5</v>
+        <v>80</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-130.5</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Gebühren</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>200</v>
+        <v>5</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-200</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>101.85</v>
+        <v>130.5</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-101.85</v>
+        <v>-130.5</v>
       </c>
     </row>
     <row r="13">
@@ -1261,17 +1233,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>79.90000000000001</v>
+        <v>200</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-79.90000000000001</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="14">
@@ -1282,79 +1254,121 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>51.8</v>
+        <v>101.85</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-51.8</v>
+        <v>-101.85</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Nebenkosten</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>1774</v>
+        <v>51.8</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-1774</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Öffentlicher Verkehr</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Nebenkosten</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Kommunikation</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="4" t="n">
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4" t="n">
         <v>51.6</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E19" s="4" t="n">
         <v>-51.6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Extends Twint send money parser to also be able to handle transaction where the sender is not mentioned. Added example rule for sharing costs of a meal using Twint.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>2990.49</v>
+        <v>3029.16</v>
       </c>
     </row>
     <row r="8">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5763.810000000001</v>
+        <v>5725.140000000001</v>
       </c>
     </row>
     <row r="11">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>1825.6</v>
+        <v>1844.27</v>
       </c>
     </row>
     <row r="24">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>130.5</v>
+        <v>150.5</v>
       </c>
     </row>
     <row r="28">
@@ -898,10 +898,10 @@
         <v>0</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1825.6</v>
+        <v>1844.27</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>-1825.6</v>
+        <v>-1844.27</v>
       </c>
     </row>
     <row r="8">
@@ -962,10 +962,10 @@
         <v>0</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>130.5</v>
+        <v>150.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>-130.5</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="12">
@@ -1219,10 +1219,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>130.5</v>
+        <v>150.5</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-130.5</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="13">
@@ -1366,10 +1366,10 @@
         <v>0</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>51.6</v>
+        <v>70.27</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-51.6</v>
+        <v>-70.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Detects money received over Twint. Categorizes them as "Rückerstattungen".
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -202,12 +202,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$14:$A$15</f>
+              <f>'Overview'!$A$14:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$14:$B$15</f>
+              <f>'Overview'!$B$14:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -250,7 +250,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!B22</f>
+              <f>'Overview'!B23</f>
             </strRef>
           </tx>
           <spPr>
@@ -260,12 +260,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$23:$A$30</f>
+              <f>'Overview'!$A$24:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$23:$B$30</f>
+              <f>'Overview'!$B$24:$B$31</f>
             </numRef>
           </val>
         </ser>
@@ -309,7 +309,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -636,7 +636,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: data/reference (1 categorized file(s))</t>
+          <t>Source: data/reference (2 categorized file(s))</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>8754.300000000001</v>
+        <v>8755.300000000001</v>
       </c>
     </row>
     <row r="7">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5725.140000000001</v>
+        <v>5726.140000000001</v>
       </c>
     </row>
     <row r="11">
@@ -716,102 +716,112 @@
         <v>1787.95</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rückerstattungen</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Expenses by Category</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Amount (CHF)</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>1844.27</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>23.95</v>
+        <v>1844.27</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Überträge</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>433.55</v>
+        <v>23.95</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>382.59</v>
+        <v>433.55</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>150.5</v>
+        <v>382.59</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>150.5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>85</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n">
+      <c r="B31" s="4" t="n">
         <v>12.4</v>
       </c>
     </row>
@@ -827,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -846,7 +856,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>January 2025</t>
         </is>
       </c>
     </row>
@@ -875,144 +885,189 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Rückerstattungen</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>6966.35</v>
+        <v>1</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>1844.27</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>-1844.27</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Überträge</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>1787.95</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>23.95</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>1764</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>433.55</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>-433.55</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>382.59</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>-382.59</v>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>150.5</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>-150.5</v>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>85</v>
+        <v>1844.27</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>-85</v>
+        <v>-1844.27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Überträge</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>1787.95</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>433.55</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>-433.55</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>382.59</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>-382.59</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>-150.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>-85</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="4" t="n">
+      <c r="B20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="4" t="n">
         <v>12.4</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D20" s="4" t="n">
         <v>-12.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Detects online purchases using PF eFinance. Adds a rule for example merchant, that categorizes as "Wohnen / Haushalt".
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>3029.16</v>
+        <v>3043.06</v>
       </c>
     </row>
     <row r="8">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5726.140000000001</v>
+        <v>5712.240000000002</v>
       </c>
     </row>
     <row r="11">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>1844.27</v>
+        <v>1858.17</v>
       </c>
     </row>
     <row r="25">
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -885,189 +885,205 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>-13.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>6966.35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1844.27</v>
+        <v>0</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>-1844.27</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>23.95</v>
+        <v>1844.27</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>1764</v>
+        <v>-1844.27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Überträge</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>433.55</v>
+        <v>23.95</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>-433.55</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>382.59</v>
+        <v>433.55</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>-382.59</v>
+        <v>-433.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>150.5</v>
+        <v>382.59</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>-150.5</v>
+        <v>-382.59</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>150.5</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>85</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>-85</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>-85</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="4" t="n">
+      <c r="B21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="4" t="n">
         <v>12.4</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D21" s="4" t="n">
         <v>-12.4</v>
       </c>
     </row>
@@ -1082,7 +1098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1102,7 +1118,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>January 2025</t>
         </is>
       </c>
     </row>
@@ -1136,294 +1152,349 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Supermärkte</t>
+          <t>Haushalt</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>200.65</v>
+        <v>13.9</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>-200.65</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Detail-Lebensmittel</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>167.29</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>-167.29</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Sonstiges Einkaufen</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>14.65</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>-14.65</v>
+        <v>-13.9</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Lohn</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bargeldbezug</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>-80</v>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Gebühren</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>-5</v>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>150.5</v>
+        <v>200.65</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-150.5</v>
+        <v>-200.65</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>200</v>
+        <v>167.29</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-200</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>101.85</v>
+        <v>14.65</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-101.85</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>79.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>-79.90000000000001</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>51.8</v>
+        <v>80</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-51.8</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Gebühren</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>5</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-96.90000000000001</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nebenkosten</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>1774</v>
+        <v>150.5</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-1774</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Familie</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>-200</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gesundheit</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>-101.85</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Styling und Wellness</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>-79.90000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sonstiges Leben</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>-51.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Öffentlicher Verkehr</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Nebenkosten</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>Kommunikation</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="4" t="n">
+      <c r="C25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4" t="n">
         <v>70.27</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E25" s="4" t="n">
         <v>-70.27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Each category now uses its own block of IDs to be able to somehow group them. Added a comment to document them, and added missing categories.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -202,12 +202,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$14:$A$16</f>
+              <f>'Overview'!$A$14:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$14:$B$16</f>
+              <f>'Overview'!$B$14:$B$15</f>
             </numRef>
           </val>
         </ser>
@@ -250,7 +250,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!B23</f>
+              <f>'Overview'!B22</f>
             </strRef>
           </tx>
           <spPr>
@@ -260,12 +260,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$24:$A$31</f>
+              <f>'Overview'!$A$23:$A$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$24:$B$31</f>
+              <f>'Overview'!$B$23:$B$29</f>
             </numRef>
           </val>
         </ser>
@@ -309,7 +309,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5712.240000000002</v>
+        <v>5712.240000000001</v>
       </c>
     </row>
     <row r="11">
@@ -709,119 +709,99 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Rückerstattungen</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>1787.95</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Rückerstattungen</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+        <v>1788.95</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Expenses by Category</t>
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Amount (CHF)</t>
-        </is>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>1893.02</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>1858.17</v>
+        <v>433.55</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>23.95</v>
+        <v>371.69</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>433.55</v>
+        <v>150.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>382.59</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>150.5</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Uncategorized</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>96.90000000000001</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Uncategorized</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n">
         <v>12.4</v>
       </c>
     </row>
@@ -969,26 +949,26 @@
         <v>0</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1844.27</v>
+        <v>1879.12</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>-1844.27</v>
+        <v>-1879.12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Überträge</t>
+          <t>Rückerstattungen</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
         <v>1787.95</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>23.95</v>
+        <v>0</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>1764</v>
+        <v>1787.95</v>
       </c>
     </row>
     <row r="16">
@@ -1017,10 +997,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>382.59</v>
+        <v>371.69</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>-382.59</v>
+        <v>-371.69</v>
       </c>
     </row>
     <row r="18">
@@ -1098,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1219,10 +1199,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>200.65</v>
+        <v>189.75</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-200.65</v>
+        <v>-189.75</v>
       </c>
     </row>
     <row r="13">
@@ -1464,7 +1444,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nebenkosten</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
@@ -1496,6 +1476,48 @@
       </c>
       <c r="E25" s="4" t="n">
         <v>-70.27</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Handwerk und Garten</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>-10.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds an overview of refunds by category.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overviews by category" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Category Analysis" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Subcategory Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -192,7 +192,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!B13</f>
+              <f>'Overviews by category'!B13</f>
             </strRef>
           </tx>
           <spPr>
@@ -202,12 +202,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$14:$A$15</f>
+              <f>'Overviews by category'!$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$14:$B$15</f>
+              <f>'Overviews by category'!$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -250,7 +250,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overview'!B22</f>
+              <f>'Overviews by category'!B35</f>
             </strRef>
           </tx>
           <spPr>
@@ -260,12 +260,70 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overview'!$A$23:$A$29</f>
+              <f>'Overviews by category'!$A$36:$A$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$23:$B$29</f>
+              <f>'Overviews by category'!$B$36:$B$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Refunds by Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overviews by category'!B57</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overviews by category'!$A$58</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overviews by category'!$B$58</f>
             </numRef>
           </val>
         </ser>
@@ -309,7 +367,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -322,6 +380,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -619,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -706,103 +786,112 @@
         <v>6966.35</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Expenses by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>1893.02</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>433.55</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>371.69</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>96.90000000000001</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Refunds by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B58" s="4" t="n">
         <v>1788.95</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Expenses by Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Amount (CHF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>1893.02</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>433.55</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>371.69</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>150.5</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Mobilität</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>96.90000000000001</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Uncategorized</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>12.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds summary sheet with an overview over all four transaction categories.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overviews by category" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Category Analysis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Subcategory Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overviews by category" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Category Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Subcategory Analysis" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,14 +42,14 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -77,18 +78,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -178,7 +180,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Income by Category</a:t>
+              <a:t>Transaction Categories Overview</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -192,7 +194,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overviews by category'!B13</f>
+              <f>'Summary'!I6</f>
             </strRef>
           </tx>
           <spPr>
@@ -202,12 +204,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$14</f>
+              <f>'Summary'!$H$7:$H$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$14</f>
+              <f>'Summary'!$I$7:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -236,7 +238,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Expenses by Category</a:t>
+              <a:t>Income by Category</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -250,7 +252,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overviews by category'!B35</f>
+              <f>'Overviews by category'!B8</f>
             </strRef>
           </tx>
           <spPr>
@@ -260,12 +262,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$36:$A$41</f>
+              <f>'Overviews by category'!$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$36:$B$41</f>
+              <f>'Overviews by category'!$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -294,6 +296,64 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Expenses by Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Overviews by category'!B30</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Overviews by category'!$A$31:$A$36</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overviews by category'!$B$31:$B$36</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Refunds by Category</a:t>
             </a:r>
           </a:p>
@@ -308,7 +368,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overviews by category'!B57</f>
+              <f>'Overviews by category'!B52</f>
             </strRef>
           </tx>
           <spPr>
@@ -318,12 +378,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$58</f>
+              <f>'Overviews by category'!$A$53</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$58</f>
+              <f>'Overviews by category'!$B$53</f>
             </numRef>
           </val>
         </ser>
@@ -343,9 +403,36 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>12</row>
+      <row>7</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -367,7 +454,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -389,7 +476,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>56</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -699,7 +786,185 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Budget Analysis Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: data/reference (2 categorized file(s))</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Overall Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Transaction Category</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Credit (CHF)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Debit (CHF)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Transaction Category</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6966.35</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>income</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>6966.35</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>3030.66</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>3030.66</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>refund</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1788.95</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>refund</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>1788.95</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>8755.300000000001</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>3030.66</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>transfer</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>transfer</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>8755.300000000001</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>3030.66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -720,177 +985,140 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Overall Summary</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Total Income:</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>8755.300000000001</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Total Expenses:</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>3043.06</v>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Income by Category</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Net (Income - Expenses):</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>5712.240000000001</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Income by Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Amount (CHF)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Einkommen</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>6966.35</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Expenses by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1893.02</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>433.55</v>
+      </c>
+    </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>Expenses by Category</t>
-        </is>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>371.69</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>150.5</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Amount (CHF)</t>
-        </is>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="n">
-        <v>1893.02</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n">
-        <v>433.55</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n">
-        <v>371.69</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="n">
-        <v>150.5</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Mobilität</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n">
-        <v>96.90000000000001</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
           <t>Finanzen</t>
         </is>
       </c>
-      <c r="B41" s="4" t="n">
+      <c r="B36" s="5" t="n">
         <v>85</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Refunds by Category</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="7" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>Amount (CHF)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B58" s="4" t="n">
+      <c r="B53" s="5" t="n">
         <v>1788.95</v>
       </c>
     </row>
@@ -900,7 +1128,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -923,29 +1151,29 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>January 2025</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
@@ -957,13 +1185,13 @@
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="4" t="n">
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n">
         <v>13.9</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>-13.9</v>
       </c>
     </row>
@@ -973,40 +1201,40 @@
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="4" t="n">
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
@@ -1018,13 +1246,13 @@
           <t>Einkommen</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>6966.35</v>
       </c>
-      <c r="C13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4" t="n">
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
         <v>6966.35</v>
       </c>
     </row>
@@ -1034,13 +1262,13 @@
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="4" t="n">
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="n">
         <v>1879.12</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>-1879.12</v>
       </c>
     </row>
@@ -1050,13 +1278,13 @@
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="5" t="n">
         <v>1787.95</v>
       </c>
-      <c r="C15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="4" t="n">
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
         <v>1787.95</v>
       </c>
     </row>
@@ -1066,13 +1294,13 @@
           <t>Leben</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="4" t="n">
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="n">
         <v>433.55</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="5" t="n">
         <v>-433.55</v>
       </c>
     </row>
@@ -1082,13 +1310,13 @@
           <t>Einkaufen</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="4" t="n">
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="n">
         <v>371.69</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>-371.69</v>
       </c>
     </row>
@@ -1098,13 +1326,13 @@
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="4" t="n">
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="n">
         <v>150.5</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="5" t="n">
         <v>-150.5</v>
       </c>
     </row>
@@ -1114,13 +1342,13 @@
           <t>Mobilität</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="4" t="n">
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="n">
         <v>96.90000000000001</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>-96.90000000000001</v>
       </c>
     </row>
@@ -1130,13 +1358,13 @@
           <t>Finanzen</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="4" t="n">
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="5" t="n">
         <v>-85</v>
       </c>
     </row>
@@ -1146,13 +1374,13 @@
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="4" t="n">
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="n">
         <v>12.4</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="5" t="n">
         <v>-12.4</v>
       </c>
     </row>
@@ -1161,7 +1389,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1185,34 +1413,34 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>January 2025</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
@@ -1229,45 +1457,45 @@
           <t>Haushalt</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>13.9</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>-13.9</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
@@ -1284,13 +1512,13 @@
           <t>Supermärkte</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
         <v>189.75</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="5" t="n">
         <v>-189.75</v>
       </c>
     </row>
@@ -1305,13 +1533,13 @@
           <t>Detail-Lebensmittel</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4" t="n">
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
         <v>167.29</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>-167.29</v>
       </c>
     </row>
@@ -1326,13 +1554,13 @@
           <t>Sonstiges Einkaufen</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="4" t="n">
+      <c r="C14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
         <v>14.65</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="5" t="n">
         <v>-14.65</v>
       </c>
     </row>
@@ -1347,13 +1575,13 @@
           <t>Lohn</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="5" t="n">
         <v>6966.35</v>
       </c>
-      <c r="D15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="4" t="n">
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
         <v>6966.35</v>
       </c>
     </row>
@@ -1368,13 +1596,13 @@
           <t>Bargeldbezug</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="4" t="n">
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="5" t="n">
         <v>-80</v>
       </c>
     </row>
@@ -1389,13 +1617,13 @@
           <t>Gebühren</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="4" t="n">
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="5" t="n">
         <v>-5</v>
       </c>
     </row>
@@ -1410,13 +1638,13 @@
           <t>Gastronomie</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="4" t="n">
+      <c r="C18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="n">
         <v>150.5</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="5" t="n">
         <v>-150.5</v>
       </c>
     </row>
@@ -1431,13 +1659,13 @@
           <t>Familie</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="4" t="n">
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>-200</v>
       </c>
     </row>
@@ -1452,13 +1680,13 @@
           <t>Gesundheit</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="4" t="n">
+      <c r="C20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n">
         <v>101.85</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="5" t="n">
         <v>-101.85</v>
       </c>
     </row>
@@ -1473,13 +1701,13 @@
           <t>Styling und Wellness</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="4" t="n">
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
         <v>79.90000000000001</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="5" t="n">
         <v>-79.90000000000001</v>
       </c>
     </row>
@@ -1494,13 +1722,13 @@
           <t>Sonstiges Leben</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="4" t="n">
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
         <v>51.8</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="5" t="n">
         <v>-51.8</v>
       </c>
     </row>
@@ -1515,13 +1743,13 @@
           <t>Öffentlicher Verkehr</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="4" t="n">
+      <c r="C23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n">
         <v>96.90000000000001</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="5" t="n">
         <v>-96.90000000000001</v>
       </c>
     </row>
@@ -1536,13 +1764,13 @@
           <t>Miete und Hypothek</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="4" t="n">
+      <c r="C24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n">
         <v>1774</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="5" t="n">
         <v>-1774</v>
       </c>
     </row>
@@ -1557,13 +1785,13 @@
           <t>Kommunikation</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="4" t="n">
+      <c r="C25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="n">
         <v>70.27</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="5" t="n">
         <v>-70.27</v>
       </c>
     </row>
@@ -1578,13 +1806,13 @@
           <t>Haushalt</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="4" t="n">
+      <c r="C26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n">
         <v>23.95</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="5" t="n">
         <v>-23.95</v>
       </c>
     </row>
@@ -1599,13 +1827,13 @@
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="4" t="n">
+      <c r="C27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Excludes transaction of transaction category "transfer" from analysis by category or subcategory.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -1150,6 +1150,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Note: Transactions with Transaction Category 'transfer' are excluded.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
@@ -1412,6 +1419,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Note: Transactions with Transaction Category 'transfer' are excluded.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adds transaction of tr category "transfer" to reference data set and tests it.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0</v>
+        <v>450</v>
       </c>
     </row>
     <row r="12">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>0</v>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>8755.300000000001</v>
+        <v>9205.300000000001</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>3030.66</v>

</xml_diff>

<commit_message>
Changed reference data of a refund from a Krankenkasse to actually go to Leben/Gesundheit.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -378,12 +378,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$53</f>
+              <f>'Overviews by category'!$A$53:$A$54</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$53</f>
+              <f>'Overviews by category'!$B$53:$B$54</f>
             </numRef>
           </val>
         </ser>
@@ -873,7 +873,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>3030.66</v>
+        <v>3049.66</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3030.66</v>
+        <v>3049.66</v>
       </c>
     </row>
     <row r="9">
@@ -915,7 +915,7 @@
         <v>8755.300000000001</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3030.66</v>
+        <v>3049.66</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>9205.300000000001</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>3030.66</v>
+        <v>3049.66</v>
       </c>
     </row>
   </sheetData>
@@ -964,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>433.55</v>
+        <v>452.55</v>
       </c>
     </row>
     <row r="33">
@@ -1115,11 +1115,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>1787.95</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
-        <v>1788.95</v>
+      <c r="B54" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1189,126 +1199,126 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>13.9</v>
+        <v>19</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>-13.9</v>
+        <v>-19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>-13.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5" t="n">
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>6966.35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>1879.12</v>
+        <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>-1879.12</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Rückerstattungen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
         <v>1787.95</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0</v>
+        <v>433.55</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>1787.95</v>
+        <v>1354.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>433.55</v>
+        <v>1879.12</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>-433.55</v>
+        <v>-1879.12</v>
       </c>
     </row>
     <row r="17">
@@ -1402,7 +1412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1463,77 +1473,77 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Familie</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>-19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Haushalt</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5" t="n">
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
         <v>13.9</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>-13.9</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Supermärkte</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>189.75</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>-189.75</v>
       </c>
     </row>
     <row r="13">
@@ -1544,17 +1554,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Detail-Lebensmittel</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>167.29</v>
+        <v>189.75</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-167.29</v>
+        <v>-189.75</v>
       </c>
     </row>
     <row r="14">
@@ -1565,59 +1575,59 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sonstiges Einkaufen</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>14.65</v>
+        <v>167.29</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-14.65</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Lohn</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>6966.35</v>
+        <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0</v>
+        <v>14.65</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>6966.35</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-80</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="17">
@@ -1628,59 +1638,59 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Gebühren</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-5</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Gebühren</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>150.5</v>
+        <v>5</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-150.5</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>200</v>
+        <v>150.5</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-200</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="20">
@@ -1695,13 +1705,13 @@
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>101.85</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-101.85</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="21">
@@ -1712,17 +1722,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>200</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="22">
@@ -1733,59 +1743,59 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>51.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-51.8</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>1774</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-1774</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -1796,17 +1806,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>70.27</v>
+        <v>1774</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-70.27</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="26">
@@ -1817,17 +1827,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>23.95</v>
+        <v>70.27</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-23.95</v>
+        <v>-70.27</v>
       </c>
     </row>
     <row r="27">
@@ -1838,16 +1848,37 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="5" t="n">
+      <c r="C28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E28" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adapted payment parser to also parse transactions with bank route.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -873,7 +873,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>3049.66</v>
+        <v>3076.36</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3049.66</v>
+        <v>3076.36</v>
       </c>
     </row>
     <row r="9">
@@ -915,7 +915,7 @@
         <v>8755.300000000001</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3049.66</v>
+        <v>3076.36</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>9205.300000000001</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>3049.66</v>
+        <v>3076.36</v>
       </c>
     </row>
   </sheetData>
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>123.6</v>
       </c>
     </row>
     <row r="36">
@@ -1144,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1199,205 +1199,221 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>19</v>
+        <v>26.7</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>-19</v>
+        <v>-26.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>13.9</v>
+        <v>19</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>-13.9</v>
+        <v>-19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>-13.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Rückerstattungen</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5" t="n">
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>6966.35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1787.95</v>
+        <v>6966.35</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>433.55</v>
+        <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>1354.4</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>1879.12</v>
+        <v>433.55</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>-1879.12</v>
+        <v>1354.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>371.69</v>
+        <v>1879.12</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>-371.69</v>
+        <v>-1879.12</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>150.5</v>
+        <v>371.69</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>-150.5</v>
+        <v>-371.69</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>150.5</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>85</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>-85</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>-85</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="5" t="n">
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="n">
         <v>12.4</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D22" s="5" t="n">
         <v>-12.4</v>
       </c>
     </row>
@@ -1412,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1494,77 +1510,77 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Privater Verkehr</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>-26.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Haushalt</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5" t="n">
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>13.9</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E8" s="5" t="n">
         <v>-13.9</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Supermärkte</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>189.75</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>-189.75</v>
       </c>
     </row>
     <row r="14">
@@ -1575,17 +1591,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Detail-Lebensmittel</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>167.29</v>
+        <v>189.75</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-167.29</v>
+        <v>-189.75</v>
       </c>
     </row>
     <row r="15">
@@ -1596,59 +1612,59 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sonstiges Einkaufen</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>14.65</v>
+        <v>167.29</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-14.65</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lohn</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
-        <v>6966.35</v>
+        <v>0</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0</v>
+        <v>14.65</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>6966.35</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-80</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="18">
@@ -1659,59 +1675,59 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gebühren</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-5</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Gebühren</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>150.5</v>
+        <v>5</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-150.5</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>101.85</v>
+        <v>150.5</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>1686.1</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="21">
@@ -1722,17 +1738,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>200</v>
+        <v>101.85</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-200</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="22">
@@ -1743,17 +1759,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>200</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="23">
@@ -1764,59 +1780,59 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>51.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-51.8</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1774</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-1774</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1827,17 +1843,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>70.27</v>
+        <v>1774</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-70.27</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="27">
@@ -1848,17 +1864,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>23.95</v>
+        <v>70.27</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-23.95</v>
+        <v>-70.27</v>
       </c>
     </row>
     <row r="28">
@@ -1869,16 +1885,37 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="5" t="n">
+      <c r="C29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E29" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added parser for purchases using Twint.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -804,7 +804,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: data/reference (2 categorized file(s))</t>
+          <t>Source: data/reference (3 categorized file(s))</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>3076.36</v>
+        <v>3079.36</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3076.36</v>
+        <v>3079.36</v>
       </c>
     </row>
     <row r="9">
@@ -915,7 +915,7 @@
         <v>8755.300000000001</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3076.36</v>
+        <v>3079.36</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         <v>9205.300000000001</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>3076.36</v>
+        <v>3079.36</v>
       </c>
     </row>
   </sheetData>
@@ -981,7 +981,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: data/reference (2 categorized file(s))</t>
+          <t>Source: data/reference (3 categorized file(s))</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>150.5</v>
+        <v>153.5</v>
       </c>
     </row>
     <row r="35">
@@ -1144,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1263,7 +1263,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>February 2025</t>
         </is>
       </c>
     </row>
@@ -1292,128 +1292,173 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>6966.35</v>
+        <v>0</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>1787.95</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>433.55</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>1354.4</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>1879.12</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>-1879.12</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>371.69</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>-371.69</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>150.5</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>-150.5</v>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Mobilität</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>96.90000000000001</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>-96.90000000000001</v>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>-85</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1787.95</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>433.55</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>1354.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>1879.12</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>-1879.12</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>371.69</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>-371.69</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>-150.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Finanzen</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>-85</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="5" t="n">
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="n">
         <v>12.4</v>
       </c>
-      <c r="D22" s="5" t="n">
+      <c r="D28" s="5" t="n">
         <v>-12.4</v>
       </c>
     </row>
@@ -1428,7 +1473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1552,7 +1597,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>March 2025</t>
+          <t>February 2025</t>
         </is>
       </c>
     </row>
@@ -1586,336 +1631,391 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Supermärkte</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>189.75</v>
+        <v>3</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-189.75</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Detail-Lebensmittel</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>167.29</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>-167.29</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Sonstiges Einkaufen</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>14.65</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>-14.65</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Lohn</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Bargeldbezug</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>-80</v>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Gebühren</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>-5</v>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>150.5</v>
+        <v>189.75</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-150.5</v>
+        <v>-189.75</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>101.85</v>
+        <v>167.29</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>1686.1</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>200</v>
+        <v>14.65</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-200</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>51.8</v>
+        <v>80</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-51.8</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Gebühren</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>5</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>1774</v>
+        <v>150.5</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-1774</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>70.27</v>
+        <v>101.85</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-70.27</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>23.95</v>
+        <v>200</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-23.95</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Styling und Wellness</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>-79.90000000000001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sonstiges Leben</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>-51.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Öffentlicher Verkehr</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Miete und Hypothek</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>1774</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>-1774</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Kommunikation</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>70.27</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>-70.27</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="5" t="n">
+      <c r="C35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E35" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve readability of categorized CSV. Values for transaction_type_detail and service translated to English. Values for transaction_type and transaction_category start with capital letter.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -378,12 +378,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$53:$A$54</f>
+              <f>'Overviews by category'!$A$53</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$53:$B$54</f>
+              <f>'Overviews by category'!$B$53</f>
             </numRef>
           </val>
         </ser>
@@ -845,7 +845,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -856,7 +856,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="I7" s="5" t="n">
@@ -866,43 +866,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>3079.36</v>
+        <v>2999.36</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3079.36</v>
+        <v>2999.36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>refund</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1788.95</v>
+        <v>1787.95</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>refund</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="I9" s="5" t="n">
-        <v>1788.95</v>
+        <v>1787.95</v>
       </c>
     </row>
     <row r="10">
@@ -912,14 +912,14 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>8755.300000000001</v>
+        <v>8754.300000000001</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>3079.36</v>
+        <v>2999.36</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>Transfer</t>
         </is>
       </c>
       <c r="I10" s="5" t="n">
@@ -929,7 +929,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>Transfer</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>9205.300000000001</v>
+        <v>9204.300000000001</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>3079.36</v>
+        <v>2999.36</v>
       </c>
     </row>
   </sheetData>
@@ -964,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>85</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -1120,16 +1120,6 @@
       </c>
       <c r="B53" s="5" t="n">
         <v>1787.95</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Rückerstattungen</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1247,7 +1237,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Rückerstattungen</t>
+          <t>Uncategorized</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -1433,33 +1423,33 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Uncategorized</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>85</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>-85</v>
+        <v>-92.40000000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>12.4</v>
+        <v>5</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>-12.4</v>
+        <v>-5</v>
       </c>
     </row>
   </sheetData>
@@ -1473,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1775,59 +1765,59 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Fees</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-80</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gebühren</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>5</v>
+        <v>150.5</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-5</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>150.5</v>
+        <v>101.85</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-150.5</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="27">
@@ -1838,17 +1828,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>101.85</v>
+        <v>200</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>1686.1</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="28">
@@ -1859,17 +1849,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>200</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-200</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1880,59 +1870,59 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>51.8</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>-51.8</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>1774</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="32">
@@ -1943,17 +1933,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>1774</v>
+        <v>70.27</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>-1774</v>
+        <v>-70.27</v>
       </c>
     </row>
     <row r="33">
@@ -1964,17 +1954,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Haushalt</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>70.27</v>
+        <v>23.95</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>-70.27</v>
+        <v>-23.95</v>
       </c>
     </row>
     <row r="34">
@@ -1985,37 +1975,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Handwerk und Garten</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>23.95</v>
+        <v>10.9</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>-23.95</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Handwerk und Garten</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="5" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E35" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adds parser for transaction representing a refund through the Postfinance Card.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -378,12 +378,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$53</f>
+              <f>'Overviews by category'!$A$53:$A$54</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$53</f>
+              <f>'Overviews by category'!$B$53:$B$54</f>
             </numRef>
           </val>
         </ser>
@@ -804,7 +804,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: data/reference (3 categorized file(s))</t>
+          <t>Source: data/reference (4 categorized file(s))</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1787.95</v>
+        <v>1887.95</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>0</v>
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="n">
-        <v>1787.95</v>
+        <v>1887.95</v>
       </c>
     </row>
     <row r="10">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>8754.300000000001</v>
+        <v>8854.300000000001</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>2999.36</v>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>9204.300000000001</v>
+        <v>9304.300000000001</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>2999.36</v>
@@ -964,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -981,7 +981,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: data/reference (3 categorized file(s))</t>
+          <t>Source: data/reference (4 categorized file(s))</t>
         </is>
       </c>
     </row>
@@ -1120,6 +1120,16 @@
       </c>
       <c r="B53" s="5" t="n">
         <v>1787.95</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1134,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1450,6 +1460,51 @@
       </c>
       <c r="D28" s="5" t="n">
         <v>-5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>April 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1463,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1988,6 +2043,61 @@
         <v>-10.9</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>April 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Reisen und Erleben</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Couple of visual fixed to ensure all headers are the same size and content starts on the same row in every sheet.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,10 +46,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -89,7 +85,6 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -252,7 +247,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overviews by category'!B8</f>
+              <f>'Overviews by category'!B7</f>
             </strRef>
           </tx>
           <spPr>
@@ -262,12 +257,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$9</f>
+              <f>'Overviews by category'!$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$9</f>
+              <f>'Overviews by category'!$B$8</f>
             </numRef>
           </val>
         </ser>
@@ -310,7 +305,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overviews by category'!B30</f>
+              <f>'Overviews by category'!B29</f>
             </strRef>
           </tx>
           <spPr>
@@ -320,12 +315,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$31:$A$36</f>
+              <f>'Overviews by category'!$A$30:$A$35</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$31:$B$36</f>
+              <f>'Overviews by category'!$B$30:$B$35</f>
             </numRef>
           </val>
         </ser>
@@ -368,7 +363,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Overviews by category'!B52</f>
+              <f>'Overviews by category'!B51</f>
             </strRef>
           </tx>
           <spPr>
@@ -378,12 +373,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$53:$A$54</f>
+              <f>'Overviews by category'!$A$52:$A$53</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$53:$B$54</f>
+              <f>'Overviews by category'!$B$52:$B$53</f>
             </numRef>
           </val>
         </ser>
@@ -432,7 +427,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>7</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -454,7 +449,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>29</row>
+      <row>28</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -476,7 +471,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>50</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5040000" cy="3600000"/>
@@ -786,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -808,51 +803,40 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Overall Summary</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Transaction Category</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Transaction Category</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Credit (CHF)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Debit (CHF)</t>
         </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Transaction Category</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Amount (CHF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -866,14 +850,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>2999.36</v>
+        <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -887,14 +871,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1887.95</v>
+        <v>0</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0</v>
+        <v>2999.36</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -906,16 +890,16 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>8854.300000000001</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>2999.36</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Refund</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1887.95</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -926,29 +910,42 @@
         <v>450</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>8854.300000000001</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>2999.36</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Transfer</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B13" s="5" t="n">
         <v>450</v>
       </c>
-      <c r="C12" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B15" s="7" t="n">
         <v>9304.300000000001</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C15" s="7" t="n">
         <v>2999.36</v>
       </c>
     </row>
@@ -964,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -985,150 +982,150 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Income by Category</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Einkommen</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>6966.35</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Expenses by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Amount (CHF)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Expenses by Category</t>
-        </is>
-      </c>
-    </row>
     <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Amount (CHF)</t>
-        </is>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1893.02</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1893.02</v>
+        <v>452.55</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>452.55</v>
+        <v>371.69</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>371.69</v>
+        <v>153.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>153.5</v>
+        <v>123.6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>123.6</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Finanzen</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>Refunds by Category</t>
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Amount (CHF)</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>Amount (CHF)</t>
-        </is>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>1787.95</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>1787.95</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1144,7 +1141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1154,7 +1151,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Category Analysis</t>
         </is>
@@ -1167,343 +1164,343 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>January 2025</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Mobilität</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>-26.7</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>-19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>13.9</v>
+        <v>26.7</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>-13.9</v>
+        <v>-26.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>-13.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Uncategorized</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B11" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="5" t="n">
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>February 2025</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="5" t="n">
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D17" s="5" t="n">
         <v>-3</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Einkommen</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>6966.35</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>1787.95</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>433.55</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>1354.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1879.12</v>
+        <v>0</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>-1879.12</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>371.69</v>
+        <v>433.55</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>-371.69</v>
+        <v>1354.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>150.5</v>
+        <v>1879.12</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>-150.5</v>
+        <v>-1879.12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>371.69</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-371.69</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>92.40000000000001</v>
+        <v>150.5</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>-92.40000000000001</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>-96.90000000000001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Uncategorized</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>-92.40000000000001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Finanzen</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="5" t="n">
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D30" s="5" t="n">
         <v>-5</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>April 2025</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n">
+      <c r="B36" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="C34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="5" t="n">
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1518,7 +1515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1529,7 +1526,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Subcategory Analysis</t>
         </is>
@@ -1542,232 +1539,190 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>January 2025</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Leben</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Familie</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>-19</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Mobilität</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Privater Verkehr</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>-26.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Leben</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Familie</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>-19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mobilität</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Privater Verkehr</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>-26.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Wohnen</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Haushalt</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="5" t="n">
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>13.9</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E10" s="5" t="n">
         <v>-13.9</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>February 2025</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Gastronomie</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5" t="n">
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E16" s="5" t="n">
         <v>-3</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>March 2025</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Supermärkte</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>189.75</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>-189.75</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Einkaufen</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Detail-Lebensmittel</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>167.29</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>-167.29</v>
       </c>
     </row>
     <row r="22">
@@ -1778,122 +1733,122 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sonstiges Einkaufen</t>
+          <t>Supermärkte</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>14.65</v>
+        <v>189.75</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-14.65</v>
+        <v>-189.75</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Lohn</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>6966.35</v>
+        <v>0</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>0</v>
+        <v>167.29</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>6966.35</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Einkaufen</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Fees</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>5</v>
+        <v>14.65</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-5</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>150.5</v>
+        <v>0</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-150.5</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Fees</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>101.85</v>
+        <v>5</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>1686.1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>200</v>
+        <v>150.5</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-200</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="28">
@@ -1904,17 +1859,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>101.85</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="29">
@@ -1925,80 +1880,80 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>51.8</v>
+        <v>200</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>-51.8</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>1774</v>
+        <v>51.8</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-1774</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>70.27</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>-70.27</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="33">
@@ -2009,17 +1964,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>23.95</v>
+        <v>1774</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>-23.95</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="34">
@@ -2030,71 +1985,113 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>Kommunikation</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>70.27</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>-70.27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="5" t="n">
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="E36" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>April 2025</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Reisen und Erleben</t>
         </is>
       </c>
-      <c r="C40" s="5" t="n">
+      <c r="C42" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="D40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="5" t="n">
+      <c r="D42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="5" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated reference xlsx for latest ref dataset.
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -373,12 +373,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$52:$A$53</f>
+              <f>'Overviews by category'!$A$52:$A$54</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$52:$B$53</f>
+              <f>'Overviews by category'!$B$52:$B$54</f>
             </numRef>
           </val>
         </ser>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>2999.36</v>
+        <v>3079.36</v>
       </c>
     </row>
     <row r="9">
@@ -878,7 +878,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>2999.36</v>
+        <v>3079.36</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="n">
-        <v>1887.95</v>
+        <v>1888.95</v>
       </c>
     </row>
     <row r="10">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1887.95</v>
+        <v>1888.95</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>0</v>
@@ -917,10 +917,10 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>8854.300000000001</v>
+        <v>8855.300000000001</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>2999.36</v>
+        <v>3079.36</v>
       </c>
     </row>
     <row r="13">
@@ -943,10 +943,10 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>9304.300000000001</v>
+        <v>9305.300000000001</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>2999.36</v>
+        <v>3079.36</v>
       </c>
     </row>
   </sheetData>
@@ -961,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
     </row>
     <row r="49">
@@ -1127,6 +1127,16 @@
       </c>
       <c r="B53" s="5" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Rückerstattungen</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1244,7 +1254,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Rückerstattungen</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
@@ -1430,33 +1440,33 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Uncategorized</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>92.40000000000001</v>
+        <v>85</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>-92.40000000000001</v>
+        <v>-85</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Uncategorized</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C30" s="5" t="n">
-        <v>5</v>
+        <v>12.4</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>-5</v>
+        <v>-12.4</v>
       </c>
     </row>
     <row r="33">
@@ -1515,7 +1525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1817,59 +1827,59 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fees</t>
+          <t>Cash Withdrawal</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-5</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Fees</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>150.5</v>
+        <v>5</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-150.5</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>101.85</v>
+        <v>150.5</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1686.1</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="29">
@@ -1880,17 +1890,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>200</v>
+        <v>101.85</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>-200</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="30">
@@ -1901,17 +1911,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>200</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="31">
@@ -1922,59 +1932,59 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>51.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-51.8</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>1774</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>-1774</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="34">
@@ -1985,17 +1995,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>70.27</v>
+        <v>1774</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>-70.27</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="35">
@@ -2006,17 +2016,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>23.95</v>
+        <v>70.27</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>-23.95</v>
+        <v>-70.27</v>
       </c>
     </row>
     <row r="36">
@@ -2027,71 +2037,92 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>Haushalt</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>-23.95</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Wohnen</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>Handwerk und Garten</t>
         </is>
       </c>
-      <c r="C36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="5" t="n">
+      <c r="C37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="n">
         <v>10.9</v>
       </c>
-      <c r="E36" s="5" t="n">
+      <c r="E37" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>April 2025</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Reisen und Erleben</t>
         </is>
       </c>
-      <c r="C42" s="5" t="n">
+      <c r="C43" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="D42" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="5" t="n">
+      <c r="D43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="5" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adds "counterparty" and "counterparty_iban" to the "scope" of notification filters.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/data/reference/output/dataset.analysis.xlsx
+++ b/data/reference/output/dataset.analysis.xlsx
@@ -257,12 +257,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$8</f>
+              <f>'Overviews by category'!$A$8:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$8</f>
+              <f>'Overviews by category'!$B$8:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -315,12 +315,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Overviews by category'!$A$30:$A$35</f>
+              <f>'Overviews by category'!$A$30:$A$36</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overviews by category'!$B$30:$B$35</f>
+              <f>'Overviews by category'!$B$30:$B$36</f>
             </numRef>
           </val>
         </ser>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>6966.35</v>
+        <v>11166.35</v>
       </c>
     </row>
     <row r="8">
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6966.35</v>
+        <v>11166.35</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>0</v>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="n">
-        <v>3079.36</v>
+        <v>3090.46</v>
       </c>
     </row>
     <row r="9">
@@ -878,7 +878,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>3079.36</v>
+        <v>3090.46</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -917,10 +917,10 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>8855.300000000001</v>
+        <v>13055.3</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>3079.36</v>
+        <v>3090.46</v>
       </c>
     </row>
     <row r="13">
@@ -943,10 +943,10 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>9305.300000000001</v>
+        <v>13505.3</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>3079.36</v>
+        <v>3090.46</v>
       </c>
     </row>
   </sheetData>
@@ -1011,6 +1011,16 @@
         <v>6966.35</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Beispiel</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4200</v>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -1037,7 +1047,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1893.02</v>
+        <v>1879.12</v>
       </c>
     </row>
     <row r="31">
@@ -1088,6 +1098,16 @@
       </c>
       <c r="B35" s="5" t="n">
         <v>85</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Beispiel</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="49">
@@ -1151,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1238,7 +1258,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wohnen</t>
+          <t>Uncategorized</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -1501,16 +1521,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Beispiel</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>4175</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B37" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="C36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="5" t="n">
+      <c r="C37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1525,7 +1561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1625,114 +1661,114 @@
         <v>-26.7</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Haushalt</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>-13.9</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>February 2025</t>
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Freizeit</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Gastronomie</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>March 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Credit in CHF</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Debit in CHF</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Net in CHF</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Freizeit</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Gastronomie</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>March 2025</t>
-        </is>
-      </c>
-    </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Subcategory</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Credit in CHF</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Debit in CHF</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Net in CHF</t>
-        </is>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Einkaufen</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Supermärkte</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>189.75</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>-189.75</v>
       </c>
     </row>
     <row r="22">
@@ -1743,17 +1779,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Supermärkte</t>
+          <t>Detail-Lebensmittel</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>189.75</v>
+        <v>167.29</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-189.75</v>
+        <v>-167.29</v>
       </c>
     </row>
     <row r="23">
@@ -1764,59 +1800,59 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Detail-Lebensmittel</t>
+          <t>Sonstiges Einkaufen</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>167.29</v>
+        <v>14.65</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-167.29</v>
+        <v>-14.65</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Einkaufen</t>
+          <t>Einkommen</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sonstiges Einkaufen</t>
+          <t>Lohn</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>0</v>
+        <v>6966.35</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>14.65</v>
+        <v>0</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>-14.65</v>
+        <v>6966.35</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Einkommen</t>
+          <t>Finanzen</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Lohn</t>
+          <t>Bargeldbezug</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>6966.35</v>
+        <v>0</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>6966.35</v>
+        <v>-80</v>
       </c>
     </row>
     <row r="26">
@@ -1827,59 +1863,59 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bargeldbezug</t>
+          <t>Fees</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-80</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Finanzen</t>
+          <t>Freizeit</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Fees</t>
+          <t>Gastronomie</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>5</v>
+        <v>150.5</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-5</v>
+        <v>-150.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Freizeit</t>
+          <t>Leben</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Gastronomie</t>
+          <t>Gesundheit</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>0</v>
+        <v>1787.95</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>150.5</v>
+        <v>101.85</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>-150.5</v>
+        <v>1686.1</v>
       </c>
     </row>
     <row r="29">
@@ -1890,17 +1926,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gesundheit</t>
+          <t>Familie</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
-        <v>1787.95</v>
+        <v>0</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>101.85</v>
+        <v>200</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1686.1</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="30">
@@ -1911,17 +1947,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Familie</t>
+          <t>Styling und Wellness</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>200</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>-200</v>
+        <v>-79.90000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1932,59 +1968,59 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Styling und Wellness</t>
+          <t>Sonstiges Leben</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>-79.90000000000001</v>
+        <v>-51.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Leben</t>
+          <t>Mobilität</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sonstiges Leben</t>
+          <t>Öffentlicher Verkehr</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>51.8</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>-51.8</v>
+        <v>-96.90000000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mobilität</t>
+          <t>Wohnen</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Öffentlicher Verkehr</t>
+          <t>Miete und Hypothek</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>96.90000000000001</v>
+        <v>1774</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>-96.90000000000001</v>
+        <v>-1774</v>
       </c>
     </row>
     <row r="34">
@@ -1995,17 +2031,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Miete und Hypothek</t>
+          <t>Kommunikation</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>1774</v>
+        <v>70.27</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>-1774</v>
+        <v>-70.27</v>
       </c>
     </row>
     <row r="35">
@@ -2016,17 +2052,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kommunikation</t>
+          <t>Haushalt</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>70.27</v>
+        <v>23.95</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>-70.27</v>
+        <v>-23.95</v>
       </c>
     </row>
     <row r="36">
@@ -2037,92 +2073,113 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Haushalt</t>
+          <t>Handwerk und Garten</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>23.95</v>
+        <v>10.9</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>-23.95</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Wohnen</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Handwerk und Garten</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E37" s="5" t="n">
         <v>-10.9</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>April 2025</t>
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Subcategory</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Credit in CHF</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Debit in CHF</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Net in CHF</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Subcategory</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Credit in CHF</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Debit in CHF</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Net in CHF</t>
-        </is>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Beispiel</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Counterparty</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>4200</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Beispiel</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Counterparty IBAN</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>-25</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>Freizeit</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Reisen und Erleben</t>
         </is>
       </c>
-      <c r="C43" s="5" t="n">
+      <c r="C44" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="D43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="5" t="n">
+      <c r="D44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="5" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>